<commit_message>
got simple cpu program working
</commit_message>
<xml_diff>
--- a/Instruction Set.xlsx
+++ b/Instruction Set.xlsx
@@ -368,10 +368,10 @@
     <t>STORER rs, rd</t>
   </si>
   <si>
-    <t>Stores rt -&gt; memory[rs]</t>
-  </si>
-  <si>
-    <t>01111 rs rt XX XXX</t>
+    <t>Stores rd -&gt; memory[rs]</t>
+  </si>
+  <si>
+    <t>01111 rs XXX XX rd</t>
   </si>
   <si>
     <t>NOP</t>

</xml_diff>

<commit_message>
added comments in instruction set
</commit_message>
<xml_diff>
--- a/Instruction Set.xlsx
+++ b/Instruction Set.xlsx
@@ -209,7 +209,7 @@
     <t>STORE addr, rd</t>
   </si>
   <si>
-    <t>Store rd → memory[addr]</t>
+    <t>Store rd → memory[addr] (rd gets converted rt internally)</t>
   </si>
   <si>
     <t>00010 addr8 rd</t>
@@ -368,7 +368,7 @@
     <t>STORER rs, rd</t>
   </si>
   <si>
-    <t>Stores rd -&gt; memory[rs]</t>
+    <t>Stores rd -&gt; memory[rs] (rd gets converted to rt internally)</t>
   </si>
   <si>
     <t>01111 rs XXX XX rd</t>

</xml_diff>